<commit_message>
debuggd excel writer and de dup it
</commit_message>
<xml_diff>
--- a/output/job_matches.xlsx
+++ b/output/job_matches.xlsx
@@ -451,42 +451,38 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Avahi</t>
+          <t>Andor Tech</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Backend Developer (.Net)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.4230300486087799</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>['data science']</t>
-        </is>
-      </c>
+        <v>0.445142388343811</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5632619810?se=hArTrxod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=7ADE3D916DFB7B28B7D4636827E29074990C6CF9</t>
+          <t>https://www.adzuna.in/land/ad/5661640050?se=hhVbtNEh8RGdbZFmEUUaJA&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=712A78F055835EB7E6D62E739BEAEB3157E20596</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>UsefulBI Corporation</t>
+          <t>HiJob.work</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Backend Developer</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -495,298 +491,270 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.4182910919189453</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>0.4383375644683838</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5646173232?se=hArTrxod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=E615FF42F5EC76CDE2FEFA0D13C4CCED49B8516A</t>
+          <t>https://www.adzuna.in/land/ad/5668762756?se=hhVbtNEh8RGdbZFmEUUaJA&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=348512D7F395BF6399F51B2A44A7B0B2D41763CB</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CoffeeBeans</t>
+          <t>Best Infosystems Ltd.</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Java Backend Developer</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Chennai, Tamil Nadu</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.4104713797569275</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>['data science']</t>
-        </is>
-      </c>
+        <v>0.4347047507762909</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5644420491?se=hArTrxod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=168E8A23B728FFBD74F39482D394D4F4D89A5CC2</t>
+          <t>https://www.adzuna.in/land/ad/5255665378?se=hhVbtNEh8RGdbZFmEUUaJA&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=E630CD9A3BDBDD395CCC3DD9C1F778173A352BE7</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>L&amp;T Technology Services</t>
+          <t>SBNRI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Backend Developer</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.390001118183136</v>
+        <v>0.4316683411598206</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>['machine learning', 'deep learning', 'data science']</t>
+          <t>python, sql</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5634429049?se=hArTrxod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=C186217FB0255E861E5FE4DEBFD7A34F7B9B5E5F</t>
+          <t>https://www.adzuna.in/land/ad/5653912905?se=hhVbtNEh8RGdbZFmEUUaJA&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=7E6C3400A17FFD269C63745A48B729F262E4CD4F</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ADM</t>
+          <t>Wipro</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Backend Developer</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.385778933763504</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>['data science']</t>
-        </is>
-      </c>
+        <v>0.4169652760028839</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5602872372?se=hArTrxod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=A3A2B15D243C834C2874221700BAD122E542A47B</t>
+          <t>https://www.adzuna.in/land/ad/5644421078?se=hhVbtNEh8RGdbZFmEUUaJA&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=30E76782BE04F22833B2A0DBB8882B588B73A07E</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CoffeeBeans</t>
+          <t>Synechron</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.3753179311752319</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>['data science']</t>
-        </is>
-      </c>
+        <v>0.4047111868858337</v>
+      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5654936383?se=hArTrxod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=E99096FDA4B28B6C259F16403C5F649D81B47B91</t>
+          <t>https://www.adzuna.in/land/ad/5643596031?se=9IN_s9Eh8RGdbZFmEUUaJA&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=64E91A8225E0AE0E3076C3F76C9C873FC8C97129</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>L&amp;T Technology Services</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Backend Developer</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Pune, Maharashtra</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.3703262805938721</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>['python', 'sql']</t>
-        </is>
-      </c>
+        <v>0.4036413729190826</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5646173811?se=NKb7rhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=AD8C32A18A87884BBFB5E7C2F2F6689298DB95D6</t>
+          <t>https://www.adzuna.in/details/5653289628?utm_medium=api&amp;utm_source=2aa433cf</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Aarvi Encon</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>Backend Developer</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Coimbatore, Tamil Nadu</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.3475925922393799</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>0.4036413729190826</v>
+      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5634430486?se=NKb7rhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=386BC4A6B9CC690372BDDFCED81D781895F056A8</t>
+          <t>https://www.adzuna.in/details/5668230542?utm_medium=api&amp;utm_source=2aa433cf</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CIBC India</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Data-Cloud engineer</t>
+          <t>Backend Developer</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.3458252251148224</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>['python']</t>
-        </is>
-      </c>
+        <v>0.4036413729190826</v>
+      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5659926187?se=jjMVrhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=24DAFEA4DEE406A4C83A83962DF01A63191072EB</t>
+          <t>https://www.adzuna.in/details/5664659271?utm_medium=api&amp;utm_source=2aa433cf</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Enterprise Minds, Inc</t>
+          <t>Sutra.AI</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.3398021459579468</v>
+        <v>0.3959265351295471</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>['python', 'sql']</t>
+          <t>machine learning</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5654936325?se=NKb7rhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=C2B154328E2DB414EEFE36EBBF255F537C6FCA4D</t>
+          <t>https://www.adzuna.in/land/ad/5604701863?se=9IN_s9Eh8RGdbZFmEUUaJA&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=D9CD85E9E26CF66671ABAD0F3FE2D4D640734F15</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>Sutra.AI</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cloud Engineering SRE</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Delhi, India</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.324546217918396</v>
+        <v>0.3945152163505554</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>machine learning</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5661258382?se=jjMVrhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=E4DD29A4E45E63AB20833B830FCA9695F2EAAEC7</t>
+          <t>https://www.adzuna.in/land/ad/5644420338?se=9IN_s9Eh8RGdbZFmEUUaJA&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=E8E5230F5908B2484DB4DBB2BE116D021E5F8254</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Daice Labs</t>
+          <t>Deutsche Telekom Digital Labs</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -795,148 +763,136 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.3177703619003296</v>
+        <v>0.3867181539535522</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>data science</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5659850050?se=NKb7rhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=4CDF696C2006EAF9AF38D4FC0C6DF98B34FFD891</t>
+          <t>https://www.adzuna.in/land/ad/5653912961?se=9IN_s9Eh8RGdbZFmEUUaJA&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=642FECC35872DCE73AF448D9B0107E230272ED3F</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Kyndryl</t>
+          <t>DraconX</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cloud Engineering Lead</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.3132890164852142</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>0.3848387598991394</v>
+      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5661258412?se=jjMVrhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=F8DA6B5AA0429C32A81CB7449A7A645F5B775A03</t>
+          <t>https://www.adzuna.in/land/ad/5661638991?se=FLErtdEh8RGtO7evCkxc9g&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=70B41A5D7EB0B79B0DB4A1BD98FE8629C7389CBF</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Albertsons Companies India</t>
+          <t>AccelEdge</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.3092997372150421</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>['machine learning']</t>
-        </is>
-      </c>
+        <v>0.3643521964550018</v>
+      </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5526832360?se=hArTrxod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=05E6A2738D4A48C7118C042538EA0BAD04D9074C</t>
+          <t>https://www.adzuna.in/land/ad/5663457437?se=9IN_s9Eh8RGdbZFmEUUaJA&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=4FF6AEF7CF2663DCB1D35857A15DB8016A529294</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Evernorth</t>
+          <t>Upbott Consulting, Inc</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cloud Engineering Lead Analyst</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>India</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.2845425009727478</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>0.3641796410083771</v>
+      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/4963670559?se=jjMVrhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=1E53198744785181E551327BA8E74F1477FC4500</t>
+          <t>https://www.adzuna.in/land/ad/5653909479?se=9IN_s9Eh8RGdbZFmEUUaJA&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=C9B031A095DEFB21053A3BCDA23FD78F614BAACD</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Canvendor</t>
+          <t>L&amp;T Technology Services</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.2740249335765839</v>
+        <v>0.3443262577056885</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>python, sql</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5653909936?se=hArTrxod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=7F7FA1998A4684D48E2EA0A9C77D1EF630A10862</t>
+          <t>https://www.adzuna.in/land/ad/5646173811?se=FLErtdEh8RGtO7evCkxc9g&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=AD8C32A18A87884BBFB5E7C2F2F6689298DB95D6</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Persistent Systems</t>
+          <t>Triaxa - FZCO</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>QA Networking Cloud Engineer</t>
+          <t>Backend Developer</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -945,83 +901,79 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.2647719979286194</v>
+        <v>0.3367191255092621</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>['python', 'aws']</t>
+          <t>kubernetes</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5632619653?se=jjMVrhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=D065A8571D76F043D56054E5AC82D9ECA60A6BA4</t>
+          <t>https://www.adzuna.in/land/ad/5656233316?se=hhVbtNEh8RGdbZFmEUUaJA&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=387E67CD6B58E77FDB464AA6AE38F1CF8DA3A40B</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Warner Bros. Discovery</t>
+          <t>QX Labs</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cloud Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.2584474682807922</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>0.3333489894866943</v>
+      </c>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5661259048?se=jjMVrhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=BB40B8517E4DF49D6CAD21751FB08CDC8FE57986</t>
+          <t>https://www.adzuna.in/land/ad/5460592900?se=9IN_s9Eh8RGdbZFmEUUaJA&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=5E0C0B6098946ACEDB232A8098A5792754CDAD16</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pearson</t>
+          <t>Enterprise Minds, Inc</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Cloud Engineer III</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Bangalore, Karnataka</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.2575602233409882</v>
+        <v>0.3278641104698181</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>['python']</t>
+          <t>python, sql</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5659930663?se=jjMVrhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=2CCC1F92AF53C71B0762B3056CB508453D69D074</t>
+          <t>https://www.adzuna.in/land/ad/5654936325?se=FLErtdEh8RGtO7evCkxc9g&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=C2B154328E2DB414EEFE36EBBF255F537C6FCA4D</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>The Briminc Softech</t>
+          <t>Daice Labs</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1035,28 +987,24 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.2507449388504028</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>0.3070492744445801</v>
+      </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5659120704?se=NKb7rhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=D1D680C84C636419E28DD04E2716B7E09B21BD32</t>
+          <t>https://www.adzuna.in/land/ad/5659850050?se=FLErtdEh8RGtO7evCkxc9g&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=4CDF696C2006EAF9AF38D4FC0C6DF98B34FFD891</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Williams-Sonoma, Inc.</t>
+          <t>ZFunds</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Junior Backend Developer</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1065,118 +1013,110 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.2482439875602722</v>
+        <v>0.292308896780014</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>node</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5635145202?se=hArTrxod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=1F60B49BBD36CD51D2CC8ADF1F3CA402C4F448EA</t>
+          <t>https://www.adzuna.in/land/ad/5648684675?se=hhVbtNEh8RGdbZFmEUUaJA&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=23568411070AB7E9C105046469BF9B70BE93EA92</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>KPI Partners</t>
+          <t>Kumaran Systems</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Data Analyst</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>Chennai, Tamil Nadu</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.2480090707540512</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>0.2751333117485046</v>
+      </c>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5647268524?se=NKb7rhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=D7DBBE578E2365631ED2FCBDDA1A00CA8752A98B</t>
+          <t>https://www.adzuna.in/land/ad/5663457269?se=9IN_s9Eh8RGdbZFmEUUaJA&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=EF37F2CA058C5B1D4A4901D5DBD43F6AB919B659</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NTT America, Inc.</t>
+          <t>Cayuse Holdings</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Azure Cloud Engineer</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Hyderabad, Telangana</t>
+          <t>New Delhi, Delhi</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.245963528752327</v>
+        <v>0.2652990520000458</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>[]</t>
+          <t>data science</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5659930639?se=jjMVrhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=24DD8936442051B22D9B82824FE91C069367D514</t>
+          <t>https://www.adzuna.in/details/5453413781?utm_medium=api&amp;utm_source=2aa433cf</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Solytics Partners</t>
+          <t>Volante Technologies</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Data Scientist</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.2436017990112305</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>['python', 'data science']</t>
-        </is>
-      </c>
+        <v>0.2476368844509125</v>
+      </c>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5657085601?se=hArTrxod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=1FB9B75436F88FCCC0D46D99B8B5DE8A5A802500</t>
+          <t>https://www.adzuna.in/land/ad/5653911606?se=FLErtdEh8RGtO7evCkxc9g&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=9603A1EA80AE1371988E21BF5105C29F4F5128E5</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>McDonalds in India</t>
+          <t>Lyric</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Cloud Engineer III</t>
+          <t>AI Engineer</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1185,23 +1125,19 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.2392179667949677</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>0.2334470897912979</v>
+      </c>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5635687417?se=jjMVrhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=4C6BCE830D4FF57DDD9662FB4043B58A643517B0</t>
+          <t>https://www.adzuna.in/details/5488837869?utm_medium=api&amp;utm_source=2aa433cf</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Enterprise Minds, Inc</t>
+          <t>Aarvi Encon</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1211,27 +1147,23 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Bangalore, Karnataka</t>
+          <t>Coimbatore, Tamil Nadu</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.2386408597230911</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>0.2283729314804077</v>
+      </c>
+      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5627769503?se=NKb7rhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=2D8C9163A9A9435E312101019FE90AC6DCF0FADD</t>
+          <t>https://www.adzuna.in/land/ad/5634430486?se=FLErtdEh8RGtO7evCkxc9g&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=386BC4A6B9CC690372BDDFCED81D781895F056A8</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Volante Technologies</t>
+          <t>Cornerstone onDemand</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1245,23 +1177,19 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.2307513952255249</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>0.2243597209453583</v>
+      </c>
+      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5653911606?se=NKb7rhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=9603A1EA80AE1371988E21BF5105C29F4F5128E5</t>
+          <t>https://www.adzuna.in/details/5637668856?utm_medium=api&amp;utm_source=2aa433cf</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Vardhman Electronics Pvt. Ltd</t>
+          <t>Cornerstone onDemand</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1271,20 +1199,16 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>New Delhi, Delhi</t>
+          <t>Pune, Maharashtra</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.2280731350183487</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>0.2243597209453583</v>
+      </c>
+      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5622178537?se=NKb7rhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=AFBD3A4AE875A4C8A174043A5B02F8188C0C2D05</t>
+          <t>https://www.adzuna.in/details/5637668857?utm_medium=api&amp;utm_source=2aa433cf</t>
         </is>
       </c>
     </row>
@@ -1305,46 +1229,42 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.2152840942144394</v>
+        <v>0.1971527636051178</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>['python']</t>
+          <t>python</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5642415932?se=NKb7rhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=D4CFB2297CB556F6C259BD30E85A87AA1F1E02C7</t>
+          <t>https://www.adzuna.in/land/ad/5642415932?se=FLErtdEh8RGtO7evCkxc9g&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=D4CFB2297CB556F6C259BD30E85A87AA1F1E02C7</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Ford Motor Company</t>
+          <t>KPI Partners</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Cloud Engineer</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Chennai, Tamil Nadu</t>
+          <t>Hyderabad, Telangana</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.1786698698997498</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>0.1654756665229797</v>
+      </c>
+      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.adzuna.in/land/ad/5661254485?se=jjMVrhod8RGHepEa_tCoWQ&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=34DFEFF5345731C8B5D17C16C73C014A9308A1D3</t>
+          <t>https://www.adzuna.in/land/ad/5647268524?se=FLErtdEh8RGtO7evCkxc9g&amp;utm_medium=api&amp;utm_source=2aa433cf&amp;v=D7DBBE578E2365631ED2FCBDDA1A00CA8752A98B</t>
         </is>
       </c>
     </row>

</xml_diff>